<commit_message>
update customer sample sheet
</commit_message>
<xml_diff>
--- a/apps/rahat-ui/public/files/sample_customer.xlsx
+++ b/apps/rahat-ui/public/files/sample_customer.xlsx
@@ -11,15 +11,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t>BDE/BDM</t>
+  </si>
   <si>
     <t>Customer Code</t>
   </si>
   <si>
     <t>Customer name</t>
-  </si>
-  <si>
-    <t>Source</t>
   </si>
   <si>
     <t>Mobile No.</t>
@@ -34,7 +34,13 @@
     <t>Region</t>
   </si>
   <si>
+    <t>Source</t>
+  </si>
+  <si>
     <t>Last purchase</t>
+  </si>
+  <si>
+    <t>John Doe</t>
   </si>
   <si>
     <t>NVG21702</t>
@@ -47,6 +53,9 @@
   </si>
   <si>
     <t>West</t>
+  </si>
+  <si>
+    <t>PRIMARY</t>
   </si>
 </sst>
 </file>
@@ -83,40 +92,32 @@
       <patternFill patternType="lightGray"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border/>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -336,24 +337,26 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="32.71"/>
-    <col customWidth="1" min="2" max="3" width="36.0"/>
-    <col customWidth="1" min="4" max="4" width="30.71"/>
+    <col customWidth="1" min="1" max="1" width="13.29"/>
+    <col customWidth="1" min="2" max="2" width="16.0"/>
+    <col customWidth="1" min="3" max="3" width="27.0"/>
+    <col customWidth="1" min="4" max="4" width="14.86"/>
     <col customWidth="1" min="5" max="5" width="8.71"/>
-    <col customWidth="1" min="6" max="6" width="23.29"/>
-    <col customWidth="1" min="7" max="7" width="34.0"/>
-    <col customWidth="1" min="8" max="8" width="35.29"/>
-    <col customWidth="1" min="9" max="27" width="8.71"/>
+    <col customWidth="1" min="6" max="6" width="12.57"/>
+    <col customWidth="1" min="7" max="7" width="11.57"/>
+    <col customWidth="1" min="8" max="8" width="13.0"/>
+    <col customWidth="1" min="9" max="9" width="18.0"/>
+    <col customWidth="1" min="10" max="28" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -368,35 +371,46 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="D2" s="3">
         <v>9.6364832E7</v>
       </c>
+      <c r="E2" s="4"/>
       <c r="F2" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="4">
+        <v>13</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="5">
         <v>45901.0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="H3" s="6"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
update: crm customer sample sheet
</commit_message>
<xml_diff>
--- a/apps/rahat-ui/public/files/sample_customer.xlsx
+++ b/apps/rahat-ui/public/files/sample_customer.xlsx
@@ -11,9 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>BDE/BDM</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>BDE</t>
+  </si>
+  <si>
+    <t>BDM</t>
   </si>
   <si>
     <t>Customer Code</t>
@@ -40,13 +43,16 @@
     <t>Last purchase</t>
   </si>
   <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>NVG21702</t>
-  </si>
-  <si>
-    <t>MANDIRI OPTIK (PALEM)</t>
+    <t>John Dai</t>
+  </si>
+  <si>
+    <t>John Vai</t>
+  </si>
+  <si>
+    <t>NVG21703</t>
+  </si>
+  <si>
+    <t>ANDIRI OPTIK (PALEM)</t>
   </si>
   <si>
     <t>Retail</t>
@@ -98,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -116,9 +122,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -337,16 +340,16 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="13.29"/>
-    <col customWidth="1" min="2" max="2" width="16.0"/>
-    <col customWidth="1" min="3" max="3" width="27.0"/>
-    <col customWidth="1" min="4" max="4" width="14.86"/>
-    <col customWidth="1" min="5" max="5" width="8.71"/>
-    <col customWidth="1" min="6" max="6" width="12.57"/>
-    <col customWidth="1" min="7" max="7" width="11.57"/>
-    <col customWidth="1" min="8" max="8" width="13.0"/>
-    <col customWidth="1" min="9" max="9" width="18.0"/>
-    <col customWidth="1" min="10" max="28" width="8.71"/>
+    <col customWidth="1" min="1" max="2" width="13.29"/>
+    <col customWidth="1" min="3" max="3" width="16.0"/>
+    <col customWidth="1" min="4" max="4" width="27.0"/>
+    <col customWidth="1" min="5" max="5" width="14.86"/>
+    <col customWidth="1" min="6" max="6" width="8.71"/>
+    <col customWidth="1" min="7" max="7" width="12.57"/>
+    <col customWidth="1" min="8" max="8" width="11.57"/>
+    <col customWidth="1" min="9" max="9" width="13.0"/>
+    <col customWidth="1" min="10" max="10" width="18.0"/>
+    <col customWidth="1" min="11" max="29" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -356,13 +359,13 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
@@ -371,46 +374,133 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="3">
-        <v>9.6364832E7</v>
-      </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="D2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="3">
+        <v>9.6364833E7</v>
+      </c>
+      <c r="F2" s="4"/>
       <c r="G2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="5">
-        <v>45901.0</v>
+        <v>15</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="5">
+        <v>45839.0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="H3" s="6"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="5"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="5"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="5"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="5"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="5"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="5"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="5"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="5"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>

</xml_diff>